<commit_message>
Melhora interface mobile e adiciona data de entrega
</commit_message>
<xml_diff>
--- a/static/modelo_upload.xlsx
+++ b/static/modelo_upload.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U1"/>
+  <dimension ref="A1:V1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,75 +449,80 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>DATA DE ENTREGA</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>LOCALIZACAO</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>BANCO</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>COMENTARIO BANCO</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>VIDROS</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>A/C</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>PREP</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>SERRA.</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>EXPE.</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>DESMONT</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>EL?TRICA</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>REVEST</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>BCO</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>ACESS?.</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>PLOTA.</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>LIBERA.</t>
         </is>

</xml_diff>

<commit_message>
feat: adiciona filtros por semana e entrega
</commit_message>
<xml_diff>
--- a/static/modelo_upload.xlsx
+++ b/static/modelo_upload.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R900e772272e348ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Ra095781e3f8c4923"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -28,7 +28,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="4">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -40,8 +40,13 @@
         <x:fgColor rgb="FF0F172A"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F172A"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="4">
+  <x:borders count="5">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -63,6 +68,20 @@
       </x:bottom>
     </x:border>
     <x:border>
+      <x:right style="thin">
+        <x:color rgb="FF334155"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF334155"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF334155"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FF334155"/>
+      </x:left>
       <x:right style="thin">
         <x:color rgb="FF334155"/>
       </x:right>
@@ -77,7 +96,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="16">
+  <x:cellXfs count="25">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -112,6 +131,27 @@
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -346,94 +386,98 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="27" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="19" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="12" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="24" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="12" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="12" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="12" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="12" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="12" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="12" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="14" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="14" hidden="0" customWidth="1"/>
-    <x:col min="20" max="20" width="14" hidden="0" customWidth="1"/>
-    <x:col min="21" max="21" width="12" hidden="0" customWidth="1"/>
-    <x:col min="22" max="22" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="17" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="12" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="22" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="11" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="11" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="11" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="11" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="11" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="9" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="13" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="12" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="13" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="9" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="12" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="12" t="str">
+      <x:c r="A1" s="21" t="str">
         <x:v>CHASSI</x:v>
       </x:c>
-      <x:c r="B1" s="13" t="str">
+      <x:c r="B1" s="21" t="str">
         <x:v>MMMV</x:v>
       </x:c>
-      <x:c r="C1" s="13" t="str">
+      <x:c r="C1" s="21" t="str">
         <x:v>LINHA</x:v>
       </x:c>
-      <x:c r="D1" s="13" t="str">
+      <x:c r="D1" s="21" t="str">
+        <x:v>SEMANA DE PRODUÇÃO</x:v>
+      </x:c>
+      <x:c r="E1" s="21" t="str">
         <x:v>AR CONDICIONADO</x:v>
       </x:c>
-      <x:c r="E1" s="13" t="str">
+      <x:c r="F1" s="21" t="str">
         <x:v>CJ. BCO</x:v>
       </x:c>
-      <x:c r="F1" s="13" t="str">
+      <x:c r="G1" s="21" t="str">
         <x:v>CLIENTE</x:v>
       </x:c>
-      <x:c r="G1" s="13" t="str">
+      <x:c r="H1" s="21" t="str">
         <x:v>DESTINO</x:v>
       </x:c>
-      <x:c r="H1" s="13" t="str">
+      <x:c r="I1" s="21" t="str">
         <x:v>DATA DE ENTREGA</x:v>
       </x:c>
-      <x:c r="I1" s="13" t="str">
+      <x:c r="J1" s="21" t="str">
         <x:v>LOCALIZACAO</x:v>
       </x:c>
-      <x:c r="J1" s="13" t="str">
+      <x:c r="K1" s="21" t="str">
         <x:v>BANCO</x:v>
       </x:c>
-      <x:c r="K1" s="13" t="str">
+      <x:c r="L1" s="21" t="str">
         <x:v>COMENTARIO BANCO</x:v>
       </x:c>
-      <x:c r="L1" s="13" t="str">
+      <x:c r="M1" s="21" t="str">
         <x:v>PREP</x:v>
       </x:c>
-      <x:c r="M1" s="13" t="str">
+      <x:c r="N1" s="21" t="str">
         <x:v>EXPE.</x:v>
       </x:c>
-      <x:c r="N1" s="13" t="str">
+      <x:c r="O1" s="21" t="str">
         <x:v>SERRA.</x:v>
       </x:c>
-      <x:c r="O1" s="13" t="str">
+      <x:c r="P1" s="21" t="str">
         <x:v>PLOTA.</x:v>
       </x:c>
-      <x:c r="P1" s="13" t="str">
+      <x:c r="Q1" s="21" t="str">
         <x:v>VIDROS</x:v>
       </x:c>
-      <x:c r="Q1" s="13" t="str">
+      <x:c r="R1" s="21" t="str">
         <x:v>A/C</x:v>
       </x:c>
-      <x:c r="R1" s="13" t="str">
+      <x:c r="S1" s="21" t="str">
         <x:v>DESMONT</x:v>
       </x:c>
-      <x:c r="S1" s="13" t="str">
+      <x:c r="T1" s="21" t="str">
         <x:v>REVEST</x:v>
       </x:c>
-      <x:c r="T1" s="13" t="str">
+      <x:c r="U1" s="21" t="str">
         <x:v>ELÉTRICA</x:v>
       </x:c>
-      <x:c r="U1" s="13" t="str">
+      <x:c r="V1" s="21" t="str">
         <x:v>BCO</x:v>
       </x:c>
-      <x:c r="V1" s="14" t="str">
+      <x:c r="W1" s="21" t="str">
         <x:v>ACESSÓ.</x:v>
       </x:c>
     </x:row>
@@ -1045,7 +1089,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd5b51df21004ecd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8bb0b2de9a545f5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>